<commit_message>
feat: complete all 10 products, 4 bundles, QA passed
Products 08-10 completed:
- P08: Client CRM Tracker (clients, pipeline, revenue, interactions)
- P09: Annual Habit Tracker (12 monthly grids, 8 habits, annual summary)
- P10: Project Management Board (tasks, resources, meetings)

All 10 products passed quality checks (品管阿瑞):
- File integrity, formulas, styling, charts, conditional formatting
- No #REF! errors, no empty sheets, proper naming

4 Bundle ZIPs generated:
- Personal Finance Bundle ($19.99) — P01,02,04,05
- Small Business Bundle ($24.99) — P06,07,08
- Freelancer Bundle ($14.99) — P03,05,10
- Ultimate Productivity Bundle ($39.99) — all 10

Product catalog (catalog.json) generated: 10/10 ready

https://claude.ai/code/session_01Qvfo6RebnKWrfFuU4vBbcE
</commit_message>
<xml_diff>
--- a/products/04-debt-payoff-planner/Debt_Payoff_Planner_SheetCraft.xlsx
+++ b/products/04-debt-payoff-planner/Debt_Payoff_Planner_SheetCraft.xlsx
@@ -292,6 +292,32 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFCCCC"/>
+          <bgColor rgb="00FFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFCC"/>
+          <bgColor rgb="00FFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00CCFFCC"/>
+          <bgColor rgb="00CCFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -366,7 +392,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -424,7 +449,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -890,12 +914,12 @@
           <t>DEBT PAYOFF DASHBOARD</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
+      <c r="B1" s="9" t="n"/>
+      <c r="C1" s="9" t="n"/>
+      <c r="D1" s="9" t="n"/>
+      <c r="E1" s="9" t="n"/>
+      <c r="F1" s="9" t="n"/>
+      <c r="G1" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1034,6 +1058,15 @@
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
+  <conditionalFormatting sqref="B11:B15">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00FF6384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1062,11 +1095,11 @@
           <t>DEBT INVENTORY</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
+      <c r="B1" s="9" t="n"/>
+      <c r="C1" s="9" t="n"/>
+      <c r="D1" s="9" t="n"/>
+      <c r="E1" s="9" t="n"/>
+      <c r="F1" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -1252,6 +1285,18 @@
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <conditionalFormatting sqref="D4:D8">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
+      <formula>0.15</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>0.07</formula>
+      <formula>0.1499</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="2">
+      <formula>0.07</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1278,10 +1323,10 @@
           <t>SNOWBALL METHOD (Smallest Balance First)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
+      <c r="B1" s="9" t="n"/>
+      <c r="C1" s="9" t="n"/>
+      <c r="D1" s="9" t="n"/>
+      <c r="E1" s="10" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
@@ -1481,10 +1526,10 @@
           <t>AVALANCHE METHOD (Highest Interest First)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
+      <c r="B1" s="9" t="n"/>
+      <c r="C1" s="9" t="n"/>
+      <c r="D1" s="9" t="n"/>
+      <c r="E1" s="10" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
@@ -1684,10 +1729,10 @@
           <t>PAYMENT LOG</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
+      <c r="B1" s="9" t="n"/>
+      <c r="C1" s="9" t="n"/>
+      <c r="D1" s="9" t="n"/>
+      <c r="E1" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -2304,8 +2349,8 @@
           <t>SNOWBALL vs AVALANCHE COMPARISON</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
+      <c r="B1" s="9" t="n"/>
+      <c r="C1" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -2447,7 +2492,7 @@
           <t>HOW TO USE YOUR DEBT PAYOFF PLANNER</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
+      <c r="B1" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="B3" s="30" t="inlineStr">

</xml_diff>